<commit_message>
Google Sheet template: bounded ranges for import
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01M7M8RsDuQjwxLQxhUj3swX
</commit_message>
<xml_diff>
--- a/templates/SOT-Google-Sheet.xlsx
+++ b/templates/SOT-Google-Sheet.xlsx
@@ -1058,13 +1058,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:C10"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="2" max="2"/>
     <col width="100" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -1451,7 +1452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:Q53"/>
+  <dimension ref="A1:Q53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="2" max="2"/>
@@ -1469,6 +1470,7 @@
     <col width="24" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
       <c r="B2" s="7" t="inlineStr">
         <is>
@@ -1482,6 +1484,7 @@
         <v/>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="B5" s="8" t="inlineStr">
         <is>
@@ -1511,19 +1514,19 @@
     </row>
     <row r="6">
       <c r="B6" s="10">
-        <f>COUNTA(DON!A3:A)-COUNTIF(DON!T3:T,"99*")-COUNTIF(DON!T3:T,"95*")</f>
+        <f>COUNTA(DON!A3:A1000)-COUNTIF(DON!T3:T1000,"99*")-COUNTIF(DON!T3:T1000,"95*")</f>
         <v/>
       </c>
       <c r="E6" s="11">
-        <f>IFERROR(COUNTIF(DON!AB3:AB,"Có")/(COUNTIF(DON!AB3:AB,"Có")+COUNTIF(DON!AB3:AB,"Không")),"–")</f>
+        <f>IFERROR(COUNTIF(DON!AB3:AB1000,"Có")/(COUNTIF(DON!AB3:AB1000,"Có")+COUNTIF(DON!AB3:AB1000,"Không")),"–")</f>
         <v/>
       </c>
       <c r="H6" s="11">
-        <f>IFERROR(COUNTIF(DON!AE3:AE,"&lt;=1")/COUNT(DON!AE3:AE),"–")</f>
+        <f>IFERROR(COUNTIF(DON!AE3:AE1000,"&lt;=1")/COUNT(DON!AE3:AE1000),"–")</f>
         <v/>
       </c>
       <c r="K6" s="10">
-        <f>COUNTIF(DON!W3:AA,"⚑")</f>
+        <f>COUNTIF(DON!W3:AA1000,"⚑")</f>
         <v/>
       </c>
       <c r="P6" t="inlineStr">
@@ -1532,7 +1535,7 @@
         </is>
       </c>
       <c r="Q6">
-        <f>COUNTIF(DON!T3:T,"10 Mới")</f>
+        <f>COUNTIF(DON!T3:T1000,"10 Mới")</f>
         <v/>
       </c>
     </row>
@@ -1558,7 +1561,7 @@
         </is>
       </c>
       <c r="Q7">
-        <f>COUNTIF(DON!T3:T,"20 Đã xác nhận")</f>
+        <f>COUNTIF(DON!T3:T1000,"20 Đã xác nhận")</f>
         <v/>
       </c>
     </row>
@@ -1569,7 +1572,7 @@
         </is>
       </c>
       <c r="Q8">
-        <f>COUNTIF(DON!T3:T,"30 Đã đặt NCC")</f>
+        <f>COUNTIF(DON!T3:T1000,"30 Đã đặt NCC")</f>
         <v/>
       </c>
     </row>
@@ -1600,25 +1603,25 @@
         </is>
       </c>
       <c r="Q9">
-        <f>COUNTIF(DON!T3:T,"40 NCC đã gửi")</f>
+        <f>COUNTIF(DON!T3:T1000,"40 NCC đã gửi")</f>
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="B10" s="13">
-        <f>IFERROR(COUNTA(CASE!A3:A)/COUNTA(DON!A3:A),"–")</f>
+        <f>IFERROR(COUNTA(CASE!A3:A1000)/COUNTA(DON!A3:A1000),"–")</f>
         <v/>
       </c>
       <c r="E10" s="14">
-        <f>IFERROR(MEDIAN(CASE!T3:T),"–")</f>
+        <f>IFERROR(MEDIAN(CASE!T3:T1000),"–")</f>
         <v/>
       </c>
       <c r="H10" s="13">
-        <f>IFERROR(COUNTIF(CASE!C3:C,"C7*")/COUNTA(DON!A3:A),"–")</f>
+        <f>IFERROR(COUNTIF(CASE!C3:C1000,"C7*")/COUNTA(DON!A3:A1000),"–")</f>
         <v/>
       </c>
       <c r="K10" s="15">
-        <f>SUM(CASE!S3:S)</f>
+        <f>SUM(CASE!S3:S1000)</f>
         <v/>
       </c>
       <c r="P10" t="inlineStr">
@@ -1627,7 +1630,7 @@
         </is>
       </c>
       <c r="Q10">
-        <f>COUNTIF(DON!T3:T,"50 QC đạt")</f>
+        <f>COUNTIF(DON!T3:T1000,"50 QC đạt")</f>
         <v/>
       </c>
     </row>
@@ -1653,7 +1656,7 @@
         </is>
       </c>
       <c r="Q11">
-        <f>COUNTIF(DON!T3:T,"60 Đã xuất")</f>
+        <f>COUNTIF(DON!T3:T1000,"60 Đã xuất")</f>
         <v/>
       </c>
     </row>
@@ -1664,7 +1667,7 @@
         </is>
       </c>
       <c r="Q12">
-        <f>COUNTIF(DON!T3:T,"70 Thông quan")</f>
+        <f>COUNTIF(DON!T3:T1000,"70 Thông quan")</f>
         <v/>
       </c>
     </row>
@@ -1675,7 +1678,7 @@
         </is>
       </c>
       <c r="Q13">
-        <f>COUNTIF(DON!T3:T,"80 Đang giao")</f>
+        <f>COUNTIF(DON!T3:T1000,"80 Đang giao")</f>
         <v/>
       </c>
     </row>
@@ -1686,7 +1689,7 @@
         </is>
       </c>
       <c r="Q14">
-        <f>COUNTIF(DON!T3:T,"90 Đã giao")</f>
+        <f>COUNTIF(DON!T3:T1000,"90 Đã giao")</f>
         <v/>
       </c>
     </row>
@@ -1697,7 +1700,7 @@
         </is>
       </c>
       <c r="Q15">
-        <f>COUNTIF(DON!T3:T,"95 Hủy/hoàn")</f>
+        <f>COUNTIF(DON!T3:T1000,"95 Hủy/hoàn")</f>
         <v/>
       </c>
     </row>
@@ -1708,10 +1711,11 @@
         </is>
       </c>
       <c r="Q16">
-        <f>COUNTIF(DON!T3:T,"99 Đóng")</f>
-        <v/>
-      </c>
-    </row>
+        <f>COUNTIF(DON!T3:T1000,"99 Đóng")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17"/>
     <row r="18">
       <c r="P18" s="9" t="inlineStr">
         <is>
@@ -1726,7 +1730,7 @@
         </is>
       </c>
       <c r="Q19">
-        <f>IFERROR(AVERAGE(DON!AE3:AE),0)</f>
+        <f>IFERROR(AVERAGE(DON!AE3:AE1000),0)</f>
         <v/>
       </c>
     </row>
@@ -1737,7 +1741,7 @@
         </is>
       </c>
       <c r="Q20">
-        <f>IFERROR(AVERAGE(DON!AF3:AF),0)</f>
+        <f>IFERROR(AVERAGE(DON!AF3:AF1000),0)</f>
         <v/>
       </c>
     </row>
@@ -1748,7 +1752,7 @@
         </is>
       </c>
       <c r="Q21">
-        <f>IFERROR(AVERAGE(DON!AG3:AG),0)</f>
+        <f>IFERROR(AVERAGE(DON!AG3:AG1000),0)</f>
         <v/>
       </c>
     </row>
@@ -1759,7 +1763,7 @@
         </is>
       </c>
       <c r="Q22">
-        <f>IFERROR(AVERAGE(DON!AH3:AH),0)</f>
+        <f>IFERROR(AVERAGE(DON!AH3:AH1000),0)</f>
         <v/>
       </c>
     </row>
@@ -1770,10 +1774,11 @@
         </is>
       </c>
       <c r="Q23">
-        <f>IFERROR(AVERAGE(DON!AI3:AI),0)</f>
-        <v/>
-      </c>
-    </row>
+        <f>IFERROR(AVERAGE(DON!AI3:AI1000),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24"/>
     <row r="25">
       <c r="P25" s="9" t="inlineStr">
         <is>
@@ -1788,7 +1793,7 @@
         </is>
       </c>
       <c r="Q26">
-        <f>COUNTIF(DON!W3:W,"⚑")</f>
+        <f>COUNTIF(DON!W3:W1000,"⚑")</f>
         <v/>
       </c>
     </row>
@@ -1799,7 +1804,7 @@
         </is>
       </c>
       <c r="Q27">
-        <f>COUNTIF(DON!X3:X,"⚑")</f>
+        <f>COUNTIF(DON!X3:X1000,"⚑")</f>
         <v/>
       </c>
     </row>
@@ -1810,7 +1815,7 @@
         </is>
       </c>
       <c r="Q28">
-        <f>COUNTIF(DON!Y3:Y,"⚑")</f>
+        <f>COUNTIF(DON!Y3:Y1000,"⚑")</f>
         <v/>
       </c>
     </row>
@@ -1821,7 +1826,7 @@
         </is>
       </c>
       <c r="Q29">
-        <f>COUNTIF(DON!Z3:Z,"⚑")</f>
+        <f>COUNTIF(DON!Z3:Z1000,"⚑")</f>
         <v/>
       </c>
     </row>
@@ -1832,7 +1837,7 @@
         </is>
       </c>
       <c r="Q30">
-        <f>COUNTIF(DON!AA3:AA,"⚑")</f>
+        <f>COUNTIF(DON!AA3:AA1000,"⚑")</f>
         <v/>
       </c>
     </row>
@@ -1843,7 +1848,7 @@
         </is>
       </c>
       <c r="Q31">
-        <f>COUNTIF(CASE!V3:V,"⚑")</f>
+        <f>COUNTIF(CASE!V3:V1000,"⚑")</f>
         <v/>
       </c>
     </row>
@@ -1854,7 +1859,7 @@
         </is>
       </c>
       <c r="Q32">
-        <f>COUNTIF(CASE!W3:W,"⚑")</f>
+        <f>COUNTIF(CASE!W3:W1000,"⚑")</f>
         <v/>
       </c>
     </row>
@@ -1865,10 +1870,11 @@
         </is>
       </c>
       <c r="Q33">
-        <f>COUNTIF(CASE!X3:X,"⚑")</f>
-        <v/>
-      </c>
-    </row>
+        <f>COUNTIF(CASE!X3:X1000,"⚑")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34"/>
     <row r="35">
       <c r="P35" s="9" t="inlineStr">
         <is>
@@ -1883,7 +1889,7 @@
         </is>
       </c>
       <c r="Q36">
-        <f>COUNTIF(CASE!C3:C,"C1 Hủy đơn")</f>
+        <f>COUNTIF(CASE!C3:C1000,"C1 Hủy đơn")</f>
         <v/>
       </c>
     </row>
@@ -1894,7 +1900,7 @@
         </is>
       </c>
       <c r="Q37">
-        <f>COUNTIF(CASE!C3:C,"C2 Trễ hạn")</f>
+        <f>COUNTIF(CASE!C3:C1000,"C2 Trễ hạn")</f>
         <v/>
       </c>
     </row>
@@ -1905,7 +1911,7 @@
         </is>
       </c>
       <c r="Q38">
-        <f>COUNTIF(CASE!C3:C,"C3 Hư hỏng")</f>
+        <f>COUNTIF(CASE!C3:C1000,"C3 Hư hỏng")</f>
         <v/>
       </c>
     </row>
@@ -1916,7 +1922,7 @@
         </is>
       </c>
       <c r="Q39">
-        <f>COUNTIF(CASE!C3:C,"C4 Thiếu kiện/phụ kiện")</f>
+        <f>COUNTIF(CASE!C3:C1000,"C4 Thiếu kiện/phụ kiện")</f>
         <v/>
       </c>
     </row>
@@ -1927,7 +1933,7 @@
         </is>
       </c>
       <c r="Q40">
-        <f>COUNTIF(CASE!C3:C,"C5 Sai hàng/khác mô tả")</f>
+        <f>COUNTIF(CASE!C3:C1000,"C5 Sai hàng/khác mô tả")</f>
         <v/>
       </c>
     </row>
@@ -1938,7 +1944,7 @@
         </is>
       </c>
       <c r="Q41">
-        <f>COUNTIF(CASE!C3:C,"C6 Đổi ý")</f>
+        <f>COUNTIF(CASE!C3:C1000,"C6 Đổi ý")</f>
         <v/>
       </c>
     </row>
@@ -1949,7 +1955,7 @@
         </is>
       </c>
       <c r="Q42">
-        <f>COUNTIF(CASE!C3:C,"C7 Chargeback")</f>
+        <f>COUNTIF(CASE!C3:C1000,"C7 Chargeback")</f>
         <v/>
       </c>
     </row>
@@ -1960,10 +1966,11 @@
         </is>
       </c>
       <c r="Q43">
-        <f>COUNTIF(CASE!C3:C,"C8 Bảo hành")</f>
-        <v/>
-      </c>
-    </row>
+        <f>COUNTIF(CASE!C3:C1000,"C8 Bảo hành")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44"/>
     <row r="45">
       <c r="P45" s="9" t="inlineStr">
         <is>
@@ -1978,7 +1985,7 @@
         </is>
       </c>
       <c r="Q46">
-        <f>COUNTIF(CASE!P3:P,"RC-NCC")</f>
+        <f>COUNTIF(CASE!P3:P1000,"RC-NCC")</f>
         <v/>
       </c>
     </row>
@@ -1989,7 +1996,7 @@
         </is>
       </c>
       <c r="Q47">
-        <f>COUNTIF(CASE!P3:P,"RC-PACK")</f>
+        <f>COUNTIF(CASE!P3:P1000,"RC-PACK")</f>
         <v/>
       </c>
     </row>
@@ -2000,7 +2007,7 @@
         </is>
       </c>
       <c r="Q48">
-        <f>COUNTIF(CASE!P3:P,"RC-QC")</f>
+        <f>COUNTIF(CASE!P3:P1000,"RC-QC")</f>
         <v/>
       </c>
     </row>
@@ -2011,7 +2018,7 @@
         </is>
       </c>
       <c r="Q49">
-        <f>COUNTIF(CASE!P3:P,"RC-FWD")</f>
+        <f>COUNTIF(CASE!P3:P1000,"RC-FWD")</f>
         <v/>
       </c>
     </row>
@@ -2022,7 +2029,7 @@
         </is>
       </c>
       <c r="Q50">
-        <f>COUNTIF(CASE!P3:P,"RC-LAST")</f>
+        <f>COUNTIF(CASE!P3:P1000,"RC-LAST")</f>
         <v/>
       </c>
     </row>
@@ -2033,7 +2040,7 @@
         </is>
       </c>
       <c r="Q51">
-        <f>COUNTIF(CASE!P3:P,"RC-LIST")</f>
+        <f>COUNTIF(CASE!P3:P1000,"RC-LIST")</f>
         <v/>
       </c>
     </row>
@@ -2044,7 +2051,7 @@
         </is>
       </c>
       <c r="Q52">
-        <f>COUNTIF(CASE!P3:P,"RC-CX")</f>
+        <f>COUNTIF(CASE!P3:P1000,"RC-CX")</f>
         <v/>
       </c>
     </row>
@@ -2055,7 +2062,7 @@
         </is>
       </c>
       <c r="Q53">
-        <f>COUNTIF(CASE!P3:P,"RC-CUST")</f>
+        <f>COUNTIF(CASE!P3:P1000,"RC-CUST")</f>
         <v/>
       </c>
     </row>
@@ -2297,75 +2304,75 @@
     </row>
     <row r="3">
       <c r="F3">
-        <f>ARRAYFORMULA(IF(E3:E="","",E3:E+7*IFERROR(VLOOKUP(B3:B,DS!$K$2:$M$4,2,FALSE),12)))</f>
+        <f>ARRAYFORMULA(IF(E3:E1000="","",E3:E1000+7*IFERROR(VLOOKUP(B3:B1000,DS!$K$2:$M$4,2,FALSE),12)))</f>
         <v/>
       </c>
       <c r="G3">
-        <f>ARRAYFORMULA(IF(E3:E="","",E3:E+7*IFERROR(VLOOKUP(B3:B,DS!$K$2:$M$4,3,FALSE),12)))</f>
+        <f>ARRAYFORMULA(IF(E3:E1000="","",E3:E1000+7*IFERROR(VLOOKUP(B3:B1000,DS!$K$2:$M$4,3,FALSE),12)))</f>
         <v/>
       </c>
       <c r="T3">
-        <f>ARRAYFORMULA(IF(A3:A="","",IF(R3:R&lt;&gt;"","95 Hủy/hoàn",IF(Q3:Q&lt;&gt;"","99 Đóng",IF(P3:P&lt;&gt;"","90 Đã giao",IF(O3:O&lt;&gt;"","80 Đang giao",IF(N3:N&lt;&gt;"","70 Thông quan",IF(M3:M&lt;&gt;"","60 Đã xuất",IF(L3:L&lt;&gt;"","50 QC đạt",IF(K3:K&lt;&gt;"","40 NCC đã gửi",IF(I3:I&lt;&gt;"","30 Đã đặt NCC",IF(H3:H&lt;&gt;"","20 Đã xác nhận","10 Mới"))))))))))))</f>
+        <f>ARRAYFORMULA(IF(A3:A1000="","",IF(R3:R1000&lt;&gt;"","95 Hủy/hoàn",IF(Q3:Q1000&lt;&gt;"","99 Đóng",IF(P3:P1000&lt;&gt;"","90 Đã giao",IF(O3:O1000&lt;&gt;"","80 Đang giao",IF(N3:N1000&lt;&gt;"","70 Thông quan",IF(M3:M1000&lt;&gt;"","60 Đã xuất",IF(L3:L1000&lt;&gt;"","50 QC đạt",IF(K3:K1000&lt;&gt;"","40 NCC đã gửi",IF(I3:I1000&lt;&gt;"","30 Đã đặt NCC",IF(H3:H1000&lt;&gt;"","20 Đã xác nhận","10 Mới"))))))))))))</f>
         <v/>
       </c>
       <c r="U3">
-        <f>ARRAYFORMULA(IF(T3:T="","",IFERROR(VLOOKUP(T3:T,DS!$A$2:$B$12,2,FALSE),"")))</f>
+        <f>ARRAYFORMULA(IF(T3:T1000="","",IFERROR(VLOOKUP(T3:T1000,DS!$A$2:$B$12,2,FALSE),"")))</f>
         <v/>
       </c>
       <c r="V3">
-        <f>ARRAYFORMULA(IF((T3:T="")+(LEFT(T3:T,2)="99")+(LEFT(T3:T,2)="95"),"",TODAY()-IF(R3:R&lt;&gt;"",R3:R,IF(Q3:Q&lt;&gt;"",Q3:Q,IF(P3:P&lt;&gt;"",P3:P,IF(O3:O&lt;&gt;"",O3:O,IF(N3:N&lt;&gt;"",N3:N,IF(M3:M&lt;&gt;"",M3:M,IF(L3:L&lt;&gt;"",L3:L,IF(K3:K&lt;&gt;"",K3:K,IF(I3:I&lt;&gt;"",I3:I,IF(H3:H&lt;&gt;"",H3:H,E3:E))))))))))))</f>
+        <f>ARRAYFORMULA(IF((T3:T1000="")+(LEFT(T3:T1000,2)="99")+(LEFT(T3:T1000,2)="95"),"",TODAY()-IF(R3:R1000&lt;&gt;"",R3:R1000,IF(Q3:Q1000&lt;&gt;"",Q3:Q1000,IF(P3:P1000&lt;&gt;"",P3:P1000,IF(O3:O1000&lt;&gt;"",O3:O1000,IF(N3:N1000&lt;&gt;"",N3:N1000,IF(M3:M1000&lt;&gt;"",M3:M1000,IF(L3:L1000&lt;&gt;"",L3:L1000,IF(K3:K1000&lt;&gt;"",K3:K1000,IF(I3:I1000&lt;&gt;"",I3:I1000,IF(H3:H1000&lt;&gt;"",H3:H1000,E3:E1000))))))))))))</f>
         <v/>
       </c>
       <c r="W3">
-        <f>ARRAYFORMULA(IF((E3:E&lt;&gt;"")*(I3:I="")*(R3:R=""),IF(TODAY()-E3:E&gt;1,"⚑",""),""))</f>
+        <f>ARRAYFORMULA(IF((E3:E1000&lt;&gt;"")*(I3:I1000="")*(R3:R1000=""),IF(TODAY()-E3:E1000&gt;1,"⚑",""),""))</f>
         <v/>
       </c>
       <c r="X3">
-        <f>ARRAYFORMULA(IF((J3:J&lt;&gt;"")*(K3:K="")*(R3:R=""),IF(TODAY()-J3:J&gt;2,"⚑",""),""))</f>
+        <f>ARRAYFORMULA(IF((J3:J1000&lt;&gt;"")*(K3:K1000="")*(R3:R1000=""),IF(TODAY()-J3:J1000&gt;2,"⚑",""),""))</f>
         <v/>
       </c>
       <c r="Y3">
-        <f>ARRAYFORMULA(IF((G3:G&lt;&gt;"")*(M3:M="")*(R3:R=""),IF((G3:G-TODAY()&lt;=14)*(G3:G&gt;=TODAY()),"⚑",""),""))</f>
+        <f>ARRAYFORMULA(IF((G3:G1000&lt;&gt;"")*(M3:M1000="")*(R3:R1000=""),IF((G3:G1000-TODAY()&lt;=14)*(G3:G1000&gt;=TODAY()),"⚑",""),""))</f>
         <v/>
       </c>
       <c r="Z3">
-        <f>ARRAYFORMULA(IF((G3:G&lt;&gt;"")*(P3:P="")*(R3:R=""),IF(TODAY()&gt;G3:G,"⚑",""),""))</f>
+        <f>ARRAYFORMULA(IF((G3:G1000&lt;&gt;"")*(P3:P1000="")*(R3:R1000=""),IF(TODAY()&gt;G3:G1000,"⚑",""),""))</f>
         <v/>
       </c>
       <c r="AA3">
-        <f>ARRAYFORMULA(IF((E3:E&lt;&gt;"")*(P3:P="")*(R3:R=""),IF(TODAY()-BYROW({E3:E,H3:H,M3:M,S3:S},LAMBDA(r,MAX(r)))&gt;7,"⚑",""),""))</f>
+        <f>ARRAYFORMULA(IF((E3:E1000&lt;&gt;"")*(P3:P1000="")*(R3:R1000=""),IF(TODAY()-IF(S3:S1000&gt;IF(M3:M1000&lt;&gt;"",M3:M1000,IF(H3:H1000&lt;&gt;"",H3:H1000,E3:E1000)),S3:S1000,IF(M3:M1000&lt;&gt;"",M3:M1000,IF(H3:H1000&lt;&gt;"",H3:H1000,E3:E1000)))&gt;7,"⚑",""),""))</f>
         <v/>
       </c>
       <c r="AB3">
-        <f>ARRAYFORMULA(IF((P3:P="")+(G3:G=""),"",IF(P3:P&lt;=G3:G,"Có","Không")))</f>
+        <f>ARRAYFORMULA(IF((P3:P1000="")+(G3:G1000=""),"",IF(P3:P1000&lt;=G3:G1000,"Có","Không")))</f>
         <v/>
       </c>
       <c r="AC3">
-        <f>ARRAYFORMULA(IF((P3:P="")+(E3:E=""),"",P3:P-E3:E))</f>
+        <f>ARRAYFORMULA(IF((P3:P1000="")+(E3:E1000=""),"",P3:P1000-E3:E1000))</f>
         <v/>
       </c>
       <c r="AD3">
-        <f>ARRAYFORMULA(IF(A3:A="","",COUNTIF(CASE!B3:B,A3:A)))</f>
+        <f>ARRAYFORMULA(IF(A3:A1000="","",COUNTIF(CASE!B3:B1000,A3:A1000)))</f>
         <v/>
       </c>
       <c r="AE3">
-        <f>ARRAYFORMULA(IF((I3:I="")+(E3:E=""),"",I3:I-E3:E))</f>
+        <f>ARRAYFORMULA(IF((I3:I1000="")+(E3:E1000=""),"",I3:I1000-E3:E1000))</f>
         <v/>
       </c>
       <c r="AF3">
-        <f>ARRAYFORMULA(IF((K3:K="")+(I3:I=""),"",K3:K-I3:I))</f>
+        <f>ARRAYFORMULA(IF((K3:K1000="")+(I3:I1000=""),"",K3:K1000-I3:I1000))</f>
         <v/>
       </c>
       <c r="AG3">
-        <f>ARRAYFORMULA(IF((L3:L="")+(K3:K=""),"",L3:L-K3:K))</f>
+        <f>ARRAYFORMULA(IF((L3:L1000="")+(K3:K1000=""),"",L3:L1000-K3:K1000))</f>
         <v/>
       </c>
       <c r="AH3">
-        <f>ARRAYFORMULA(IF((M3:M="")+(L3:L=""),"",M3:M-L3:L))</f>
+        <f>ARRAYFORMULA(IF((M3:M1000="")+(L3:L1000=""),"",M3:M1000-L3:L1000))</f>
         <v/>
       </c>
       <c r="AI3">
-        <f>ARRAYFORMULA(IF((P3:P="")+(M3:M=""),"",P3:P-M3:M))</f>
+        <f>ARRAYFORMULA(IF((P3:P1000="")+(M3:M1000=""),"",P3:P1000-M3:M1000))</f>
         <v/>
       </c>
     </row>
@@ -2584,35 +2591,35 @@
     </row>
     <row r="3">
       <c r="J3">
-        <f>ARRAYFORMULA(IF(I3:I="","",IF((I3:I&gt;150)+(H3:H="R4 Hoàn 100%"),"CEO",IF(I3:I&gt;50,"OPS","CX"))))</f>
+        <f>ARRAYFORMULA(IF(I3:I1000="","",IF((I3:I1000&gt;150)+(H3:H1000="R4 Hoàn 100%"),"CEO",IF(I3:I1000&gt;50,"OPS","CX"))))</f>
         <v/>
       </c>
       <c r="L3">
-        <f>ARRAYFORMULA(IF((J3:J="")+(K3:K=""),"",IF(IFERROR(MATCH(K3:K,DS!$H$2:$H$4,0),0)&gt;=IFERROR(MATCH(J3:J,DS!$H$2:$H$4,0),9),"✓","✗")))</f>
+        <f>ARRAYFORMULA(IF((J3:J1000="")+(K3:K1000=""),"",IF(IFERROR(MATCH(K3:K1000,DS!$H$2:$H$4,0),0)&gt;=IFERROR(MATCH(J3:J1000,DS!$H$2:$H$4,0),9),"✓","✗")))</f>
         <v/>
       </c>
       <c r="S3">
-        <f>ARRAYFORMULA(IF(A3:A="","",IFERROR(I3:I*1,0)-IFERROR(R3:R*1,0)))</f>
+        <f>ARRAYFORMULA(IF(A3:A1000="","",IFERROR(I3:I1000*1,0)-IFERROR(R3:R1000*1,0)))</f>
         <v/>
       </c>
       <c r="T3">
-        <f>ARRAYFORMULA(IF((E3:E="")+(F3:F=""),"",ROUND((F3:F-E3:E)*24,1)))</f>
+        <f>ARRAYFORMULA(IF((E3:E1000="")+(F3:F1000=""),"",ROUND((F3:F1000-E3:E1000)*24,1)))</f>
         <v/>
       </c>
       <c r="U3">
-        <f>ARRAYFORMULA(IF(E3:E="","",INT(IF(O3:O="",NOW(),O3:O)-E3:E)))</f>
+        <f>ARRAYFORMULA(IF(E3:E1000="","",INT(IF(O3:O1000="",NOW(),O3:O1000)-E3:E1000)))</f>
         <v/>
       </c>
       <c r="V3">
-        <f>ARRAYFORMULA(IF(E3:E="","",IF(F3:F="",IF((NOW()-E3:E)*24&gt;24,"⚑",""),IF((F3:F-E3:E)*24&gt;24,"⚑",""))))</f>
+        <f>ARRAYFORMULA(IF(E3:E1000="","",IF(F3:F1000="",IF((NOW()-E3:E1000)*24&gt;24,"⚑",""),IF((F3:F1000-E3:E1000)*24&gt;24,"⚑",""))))</f>
         <v/>
       </c>
       <c r="W3">
-        <f>ARRAYFORMULA(IF((E3:E="")+(O3:O&lt;&gt;""),"",IF(NOW()-E3:E&gt;7,"⚑","")))</f>
+        <f>ARRAYFORMULA(IF((E3:E1000="")+(O3:O1000&lt;&gt;""),"",IF(NOW()-E3:E1000&gt;7,"⚑","")))</f>
         <v/>
       </c>
       <c r="X3">
-        <f>ARRAYFORMULA(IF(L3:L="✗","⚑",""))</f>
+        <f>ARRAYFORMULA(IF(L3:L1000="✗","⚑",""))</f>
         <v/>
       </c>
     </row>

</xml_diff>